<commit_message>
Templates: remove references to the retired SAMPLE badge/ribbon, point RAID guidance at the new RAID template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/ATS_POAP_Template.xlsx
+++ b/templates/ATS_POAP_Template.xlsx
@@ -44,7 +44,7 @@
     <t xml:space="preserve">1. POAP_Config</t>
   </si>
   <si>
-    <t xml:space="preserve">Set program name, plan start/end and (optionally) a status date. Leave the status date blank to use today's date. Set Data Mode to LIVE for real data (SAMPLE shows a ribbon in the dashboard). Edit pillar/activity colours if you like (hex, no #).</t>
+    <t xml:space="preserve">Set program name, plan start/end and (optionally) a status date. Leave the status date blank to use today's date. Leave Data Mode as LIVE for real data. Edit pillar/activity colours if you like (hex, no #).</t>
   </si>
   <si>
     <t xml:space="preserve">2. POAP_Plan</t>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">LIVE</t>
   </si>
   <si>
-    <t xml:space="preserve">SAMPLE shows a ribbon in the dashboard; use LIVE for real data.</t>
+    <t xml:space="preserve">Leave as LIVE for real data (the dashboard shows no badge either way).</t>
   </si>
   <si>
     <t xml:space="preserve">PILLARS</t>

</xml_diff>